<commit_message>
bug fix for missing scale bar after stat
</commit_message>
<xml_diff>
--- a/stat/LAIs.xlsx
+++ b/stat/LAIs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au686295\GitHub\postdoc\Field-Image-Calibration\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD658041-A96E-4E26-84E0-1CE840C109EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4168EE12-BF78-4329-BA63-467877E137B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="81495" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39180" yWindow="780" windowWidth="28800" windowHeight="15285" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="glacier_algae (2)" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="51">
   <si>
     <t>Sample</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t>cc_frac</t>
+  </si>
+  <si>
+    <t>Area scraped (cm2) - approx</t>
   </si>
 </sst>
 </file>
@@ -2770,17 +2773,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87355849-A836-4308-8FB1-2EDC5A9AE78D}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.88671875" customWidth="1"/>
-    <col min="7" max="7" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2816,7 +2819,7 @@
       </c>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2849,7 +2852,7 @@
       </c>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2882,7 +2885,7 @@
       </c>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -2913,7 +2916,7 @@
       </c>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -2944,7 +2947,7 @@
       </c>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -2977,7 +2980,7 @@
       </c>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -3010,7 +3013,7 @@
       </c>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -3043,7 +3046,7 @@
       </c>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -3076,7 +3079,7 @@
       </c>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -3101,7 +3104,7 @@
       <c r="J10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -3132,7 +3135,7 @@
       </c>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -3155,7 +3158,7 @@
       <c r="J12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -3186,7 +3189,7 @@
       </c>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -3217,7 +3220,7 @@
       </c>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -3248,7 +3251,7 @@
       </c>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -3281,7 +3284,7 @@
       </c>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -3314,7 +3317,7 @@
         <v>392.26292303499861</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -3345,7 +3348,7 @@
       </c>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -3378,7 +3381,7 @@
       </c>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -3411,7 +3414,7 @@
       </c>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3444,7 +3447,7 @@
       </c>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -3477,7 +3480,7 @@
       </c>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -3500,7 +3503,7 @@
       <c r="J23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -3533,7 +3536,7 @@
       </c>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -3566,7 +3569,7 @@
       </c>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -3589,7 +3592,7 @@
       <c r="J26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -3609,7 +3612,7 @@
       <c r="J27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
@@ -3632,7 +3635,7 @@
       <c r="J28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>38</v>
       </c>
@@ -3661,7 +3664,7 @@
       </c>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -3690,7 +3693,7 @@
       </c>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>40</v>
       </c>
@@ -3719,7 +3722,7 @@
       </c>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>41</v>
       </c>
@@ -3746,7 +3749,7 @@
       </c>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>42</v>
       </c>
@@ -3782,17 +3785,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D19B3ED-559A-4604-B734-5B39E6D3177C}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.88671875" customWidth="1"/>
-    <col min="7" max="7" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3806,7 +3809,7 @@
         <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>35</v>
@@ -3828,7 +3831,7 @@
       </c>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3861,7 +3864,7 @@
       </c>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -3894,7 +3897,7 @@
       </c>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -3925,7 +3928,7 @@
       </c>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -3956,7 +3959,7 @@
       </c>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -3989,7 +3992,7 @@
       </c>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -4022,7 +4025,7 @@
       </c>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -4055,7 +4058,7 @@
       </c>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -4088,7 +4091,7 @@
       </c>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -4113,7 +4116,7 @@
       <c r="J10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -4144,7 +4147,7 @@
       </c>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -4167,7 +4170,7 @@
       <c r="J12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -4198,7 +4201,7 @@
       </c>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -4229,7 +4232,7 @@
       </c>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -4260,7 +4263,7 @@
       </c>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -4293,7 +4296,7 @@
       </c>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -4326,7 +4329,7 @@
         <v>392.26292303499861</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -4357,7 +4360,7 @@
       </c>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -4390,7 +4393,7 @@
       </c>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -4423,7 +4426,7 @@
       </c>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -4456,7 +4459,7 @@
       </c>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -4489,7 +4492,7 @@
       </c>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -4512,7 +4515,7 @@
       <c r="J23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -4545,7 +4548,7 @@
       </c>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -4578,7 +4581,7 @@
       </c>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -4601,7 +4604,7 @@
       <c r="J26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -4621,7 +4624,7 @@
       <c r="J27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
@@ -4644,7 +4647,7 @@
       <c r="J28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>38</v>
       </c>
@@ -4670,7 +4673,7 @@
       </c>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -4696,7 +4699,7 @@
       </c>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>40</v>
       </c>
@@ -4722,7 +4725,7 @@
       </c>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>41</v>
       </c>
@@ -4746,7 +4749,7 @@
       </c>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>42</v>
       </c>
@@ -4779,14 +4782,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71879878-E451-4C06-B017-0A13EE945E08}">
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.21875" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4824,7 +4827,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
@@ -4854,7 +4857,7 @@
       </c>
       <c r="L2" s="1"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>45</v>
       </c>
@@ -4884,7 +4887,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>46</v>
       </c>
@@ -4913,7 +4916,7 @@
         <v>17252.333333333332</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>43</v>
       </c>
@@ -4942,7 +4945,7 @@
         <v>9421</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>44</v>
       </c>
@@ -4971,7 +4974,7 @@
         <v>7451.333333333333</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4984,7 +4987,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -4997,7 +5000,7 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -5010,7 +5013,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -5023,7 +5026,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -5036,7 +5039,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -5049,7 +5052,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5062,7 +5065,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -5075,7 +5078,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -5088,7 +5091,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5101,7 +5104,7 @@
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5114,7 +5117,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -5127,7 +5130,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -5135,7 +5138,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5148,7 +5151,7 @@
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5161,7 +5164,7 @@
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5174,7 +5177,7 @@
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -5187,7 +5190,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -5200,7 +5203,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -5213,7 +5216,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -5226,7 +5229,7 @@
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -5239,7 +5242,7 @@
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -5252,7 +5255,7 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -5265,7 +5268,7 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -5278,7 +5281,7 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -5290,7 +5293,7 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -5298,7 +5301,7 @@
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -5311,11 +5314,11 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
     </row>

</xml_diff>